<commit_message>
acuracia e precision de ensemble total e parcial
</commit_message>
<xml_diff>
--- a/data/ibov/ibov_filtrado.xlsx
+++ b/data/ibov/ibov_filtrado.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>38376</v>
+        <v>44564</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
@@ -470,7 +470,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>38378</v>
+        <v>44565</v>
       </c>
       <c r="B3" t="n">
         <v>1</v>
@@ -484,7 +484,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>38379</v>
+        <v>44566</v>
       </c>
       <c r="B4" t="n">
         <v>1</v>
@@ -498,7 +498,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>38380</v>
+        <v>44567</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
@@ -512,7 +512,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>38383</v>
+        <v>44568</v>
       </c>
       <c r="B6" t="n">
         <v>1</v>
@@ -526,7 +526,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>38384</v>
+        <v>44571</v>
       </c>
       <c r="B7" t="n">
         <v>1</v>
@@ -540,7 +540,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>38385</v>
+        <v>44572</v>
       </c>
       <c r="B8" t="n">
         <v>1</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>38386</v>
+        <v>44573</v>
       </c>
       <c r="B9" t="n">
         <v>1</v>
@@ -568,7 +568,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>38387</v>
+        <v>44574</v>
       </c>
       <c r="B10" t="n">
         <v>1</v>
@@ -582,7 +582,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>38392</v>
+        <v>44575</v>
       </c>
       <c r="B11" t="n">
         <v>1</v>
@@ -596,7 +596,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>38393</v>
+        <v>44578</v>
       </c>
       <c r="B12" t="n">
         <v>1</v>
@@ -610,7 +610,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>38394</v>
+        <v>44579</v>
       </c>
       <c r="B13" t="n">
         <v>1</v>
@@ -624,7 +624,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>38397</v>
+        <v>44580</v>
       </c>
       <c r="B14" t="n">
         <v>1</v>
@@ -638,7 +638,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>38398</v>
+        <v>44581</v>
       </c>
       <c r="B15" t="n">
         <v>1</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>38399</v>
+        <v>44582</v>
       </c>
       <c r="B16" t="n">
         <v>1</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>38400</v>
+        <v>44585</v>
       </c>
       <c r="B17" t="n">
         <v>1</v>
@@ -680,7 +680,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>38401</v>
+        <v>44586</v>
       </c>
       <c r="B18" t="n">
         <v>1</v>
@@ -694,7 +694,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>38404</v>
+        <v>44587</v>
       </c>
       <c r="B19" t="n">
         <v>1</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>38405</v>
+        <v>44588</v>
       </c>
       <c r="B20" t="n">
         <v>1</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>38406</v>
+        <v>44589</v>
       </c>
       <c r="B21" t="n">
         <v>1</v>
@@ -736,7 +736,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>38407</v>
+        <v>44592</v>
       </c>
       <c r="B22" t="n">
         <v>1</v>
@@ -750,7 +750,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>38408</v>
+        <v>44593</v>
       </c>
       <c r="B23" t="n">
         <v>1</v>
@@ -764,7 +764,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>38411</v>
+        <v>44594</v>
       </c>
       <c r="B24" t="n">
         <v>1</v>
@@ -778,7 +778,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>38412</v>
+        <v>44595</v>
       </c>
       <c r="B25" t="n">
         <v>1</v>
@@ -792,7 +792,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>38413</v>
+        <v>44596</v>
       </c>
       <c r="B26" t="n">
         <v>1</v>
@@ -806,7 +806,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>38414</v>
+        <v>44599</v>
       </c>
       <c r="B27" t="n">
         <v>1</v>
@@ -820,7 +820,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>38415</v>
+        <v>44600</v>
       </c>
       <c r="B28" t="n">
         <v>1</v>
@@ -834,7 +834,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>38418</v>
+        <v>44601</v>
       </c>
       <c r="B29" t="n">
         <v>1</v>
@@ -848,7 +848,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>38419</v>
+        <v>44602</v>
       </c>
       <c r="B30" t="n">
         <v>1</v>
@@ -862,7 +862,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>38420</v>
+        <v>44603</v>
       </c>
       <c r="B31" t="n">
         <v>1</v>
@@ -876,7 +876,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>38421</v>
+        <v>44606</v>
       </c>
       <c r="B32" t="n">
         <v>1</v>
@@ -890,7 +890,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>38422</v>
+        <v>44607</v>
       </c>
       <c r="B33" t="n">
         <v>1</v>
@@ -904,7 +904,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>38425</v>
+        <v>44608</v>
       </c>
       <c r="B34" t="n">
         <v>1</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>38426</v>
+        <v>44609</v>
       </c>
       <c r="B35" t="n">
         <v>1</v>
@@ -932,7 +932,7 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>38427</v>
+        <v>44610</v>
       </c>
       <c r="B36" t="n">
         <v>1</v>
@@ -946,7 +946,7 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>38428</v>
+        <v>44613</v>
       </c>
       <c r="B37" t="n">
         <v>1</v>
@@ -960,7 +960,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>38429</v>
+        <v>44614</v>
       </c>
       <c r="B38" t="n">
         <v>1</v>
@@ -974,7 +974,7 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>38432</v>
+        <v>44615</v>
       </c>
       <c r="B39" t="n">
         <v>1</v>
@@ -988,7 +988,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>38433</v>
+        <v>44616</v>
       </c>
       <c r="B40" t="n">
         <v>1</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>38434</v>
+        <v>44617</v>
       </c>
       <c r="B41" t="n">
         <v>1</v>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>38435</v>
+        <v>44622</v>
       </c>
       <c r="B42" t="n">
         <v>1</v>
@@ -1030,7 +1030,7 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>38439</v>
+        <v>44623</v>
       </c>
       <c r="B43" t="n">
         <v>1</v>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>38440</v>
+        <v>44624</v>
       </c>
       <c r="B44" t="n">
         <v>1</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>38441</v>
+        <v>44627</v>
       </c>
       <c r="B45" t="n">
         <v>1</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>38442</v>
+        <v>44628</v>
       </c>
       <c r="B46" t="n">
         <v>1</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>38443</v>
+        <v>44629</v>
       </c>
       <c r="B47" t="n">
         <v>1</v>
@@ -1100,7 +1100,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>38446</v>
+        <v>44630</v>
       </c>
       <c r="B48" t="n">
         <v>1</v>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>38447</v>
+        <v>44631</v>
       </c>
       <c r="B49" t="n">
         <v>1</v>
@@ -1128,7 +1128,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>38448</v>
+        <v>44634</v>
       </c>
       <c r="B50" t="n">
         <v>1</v>
@@ -1142,7 +1142,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>38449</v>
+        <v>44635</v>
       </c>
       <c r="B51" t="n">
         <v>1</v>
@@ -1151,6 +1151,2806 @@
         <v>1</v>
       </c>
       <c r="D51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>44636</v>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>44637</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>44638</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>44641</v>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>44642</v>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>44643</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>44644</v>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>44645</v>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>44648</v>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>44649</v>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>44650</v>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>44651</v>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>44652</v>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>44655</v>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>44656</v>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>44657</v>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>44658</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>44659</v>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>44662</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>44663</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>44664</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>44665</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>44669</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>44670</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>44671</v>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>44673</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>44676</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>44677</v>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>44678</v>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>44679</v>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>44680</v>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>44683</v>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>44684</v>
+      </c>
+      <c r="B84" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>44685</v>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>44686</v>
+      </c>
+      <c r="B86" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>44687</v>
+      </c>
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>44690</v>
+      </c>
+      <c r="B88" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>44691</v>
+      </c>
+      <c r="B89" t="n">
+        <v>1</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>44692</v>
+      </c>
+      <c r="B90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>44693</v>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>44694</v>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>44697</v>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>44698</v>
+      </c>
+      <c r="B94" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>44699</v>
+      </c>
+      <c r="B95" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>44700</v>
+      </c>
+      <c r="B96" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>44701</v>
+      </c>
+      <c r="B97" t="n">
+        <v>1</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>44704</v>
+      </c>
+      <c r="B98" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>44705</v>
+      </c>
+      <c r="B99" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>44706</v>
+      </c>
+      <c r="B100" t="n">
+        <v>1</v>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>44707</v>
+      </c>
+      <c r="B101" t="n">
+        <v>1</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="n">
+        <v>44708</v>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="n">
+        <v>44711</v>
+      </c>
+      <c r="B103" t="n">
+        <v>1</v>
+      </c>
+      <c r="C103" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="n">
+        <v>44712</v>
+      </c>
+      <c r="B104" t="n">
+        <v>1</v>
+      </c>
+      <c r="C104" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="n">
+        <v>44713</v>
+      </c>
+      <c r="B105" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="n">
+        <v>44714</v>
+      </c>
+      <c r="B106" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="n">
+        <v>44715</v>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="n">
+        <v>44718</v>
+      </c>
+      <c r="B108" t="n">
+        <v>1</v>
+      </c>
+      <c r="C108" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="n">
+        <v>44719</v>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="n">
+        <v>44720</v>
+      </c>
+      <c r="B110" t="n">
+        <v>1</v>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="n">
+        <v>44721</v>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="n">
+        <v>44722</v>
+      </c>
+      <c r="B112" t="n">
+        <v>1</v>
+      </c>
+      <c r="C112" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="n">
+        <v>44725</v>
+      </c>
+      <c r="B113" t="n">
+        <v>1</v>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="n">
+        <v>44726</v>
+      </c>
+      <c r="B114" t="n">
+        <v>1</v>
+      </c>
+      <c r="C114" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="n">
+        <v>44727</v>
+      </c>
+      <c r="B115" t="n">
+        <v>1</v>
+      </c>
+      <c r="C115" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="n">
+        <v>44729</v>
+      </c>
+      <c r="B116" t="n">
+        <v>1</v>
+      </c>
+      <c r="C116" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
+        <v>44732</v>
+      </c>
+      <c r="B117" t="n">
+        <v>1</v>
+      </c>
+      <c r="C117" t="n">
+        <v>1</v>
+      </c>
+      <c r="D117" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="n">
+        <v>44733</v>
+      </c>
+      <c r="B118" t="n">
+        <v>1</v>
+      </c>
+      <c r="C118" t="n">
+        <v>1</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="n">
+        <v>44734</v>
+      </c>
+      <c r="B119" t="n">
+        <v>1</v>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
+      </c>
+      <c r="D119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="n">
+        <v>44735</v>
+      </c>
+      <c r="B120" t="n">
+        <v>1</v>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="n">
+        <v>44736</v>
+      </c>
+      <c r="B121" t="n">
+        <v>1</v>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="n">
+        <v>44739</v>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="n">
+        <v>44740</v>
+      </c>
+      <c r="B123" t="n">
+        <v>1</v>
+      </c>
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
+      <c r="D123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="n">
+        <v>44741</v>
+      </c>
+      <c r="B124" t="n">
+        <v>1</v>
+      </c>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="n">
+        <v>44742</v>
+      </c>
+      <c r="B125" t="n">
+        <v>1</v>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="n">
+        <v>44743</v>
+      </c>
+      <c r="B126" t="n">
+        <v>1</v>
+      </c>
+      <c r="C126" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
+        <v>44746</v>
+      </c>
+      <c r="B127" t="n">
+        <v>1</v>
+      </c>
+      <c r="C127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
+        <v>44747</v>
+      </c>
+      <c r="B128" t="n">
+        <v>1</v>
+      </c>
+      <c r="C128" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
+        <v>44748</v>
+      </c>
+      <c r="B129" t="n">
+        <v>1</v>
+      </c>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="n">
+        <v>44749</v>
+      </c>
+      <c r="B130" t="n">
+        <v>1</v>
+      </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="n">
+        <v>44750</v>
+      </c>
+      <c r="B131" t="n">
+        <v>1</v>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="n">
+        <v>44753</v>
+      </c>
+      <c r="B132" t="n">
+        <v>1</v>
+      </c>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="n">
+        <v>44754</v>
+      </c>
+      <c r="B133" t="n">
+        <v>1</v>
+      </c>
+      <c r="C133" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="n">
+        <v>44755</v>
+      </c>
+      <c r="B134" t="n">
+        <v>1</v>
+      </c>
+      <c r="C134" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="n">
+        <v>44756</v>
+      </c>
+      <c r="B135" t="n">
+        <v>1</v>
+      </c>
+      <c r="C135" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>44757</v>
+      </c>
+      <c r="B136" t="n">
+        <v>1</v>
+      </c>
+      <c r="C136" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>44760</v>
+      </c>
+      <c r="B137" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>44761</v>
+      </c>
+      <c r="B138" t="n">
+        <v>1</v>
+      </c>
+      <c r="C138" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="n">
+        <v>44762</v>
+      </c>
+      <c r="B139" t="n">
+        <v>1</v>
+      </c>
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="n">
+        <v>44763</v>
+      </c>
+      <c r="B140" t="n">
+        <v>1</v>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="n">
+        <v>44764</v>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="n">
+        <v>44767</v>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="n">
+        <v>44768</v>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="n">
+        <v>44769</v>
+      </c>
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="n">
+        <v>44770</v>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="n">
+        <v>44771</v>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="n">
+        <v>44774</v>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="n">
+        <v>44775</v>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="n">
+        <v>1</v>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
+        <v>44776</v>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="n">
+        <v>44777</v>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+      <c r="C150" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="n">
+        <v>44778</v>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="n">
+        <v>44781</v>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="n">
+        <v>44782</v>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="n">
+        <v>44783</v>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="n">
+        <v>44784</v>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="n">
+        <v>44785</v>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="n">
+        <v>44788</v>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="n">
+        <v>44789</v>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="n">
+        <v>44790</v>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="n">
+        <v>44791</v>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="n">
+        <v>44792</v>
+      </c>
+      <c r="B161" t="n">
+        <v>1</v>
+      </c>
+      <c r="C161" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>44795</v>
+      </c>
+      <c r="B162" t="n">
+        <v>1</v>
+      </c>
+      <c r="C162" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>44796</v>
+      </c>
+      <c r="B163" t="n">
+        <v>1</v>
+      </c>
+      <c r="C163" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>44797</v>
+      </c>
+      <c r="B164" t="n">
+        <v>1</v>
+      </c>
+      <c r="C164" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>44798</v>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>44799</v>
+      </c>
+      <c r="B166" t="n">
+        <v>1</v>
+      </c>
+      <c r="C166" t="n">
+        <v>1</v>
+      </c>
+      <c r="D166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>44802</v>
+      </c>
+      <c r="B167" t="n">
+        <v>1</v>
+      </c>
+      <c r="C167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>44803</v>
+      </c>
+      <c r="B168" t="n">
+        <v>1</v>
+      </c>
+      <c r="C168" t="n">
+        <v>1</v>
+      </c>
+      <c r="D168" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>44804</v>
+      </c>
+      <c r="B169" t="n">
+        <v>1</v>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>44805</v>
+      </c>
+      <c r="B170" t="n">
+        <v>1</v>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>44806</v>
+      </c>
+      <c r="B171" t="n">
+        <v>1</v>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>44809</v>
+      </c>
+      <c r="B172" t="n">
+        <v>1</v>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>44810</v>
+      </c>
+      <c r="B173" t="n">
+        <v>1</v>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>44812</v>
+      </c>
+      <c r="B174" t="n">
+        <v>1</v>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="n">
+        <v>44813</v>
+      </c>
+      <c r="B175" t="n">
+        <v>1</v>
+      </c>
+      <c r="C175" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="n">
+        <v>44816</v>
+      </c>
+      <c r="B176" t="n">
+        <v>1</v>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="n">
+        <v>44817</v>
+      </c>
+      <c r="B177" t="n">
+        <v>1</v>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="n">
+        <v>44818</v>
+      </c>
+      <c r="B178" t="n">
+        <v>1</v>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="n">
+        <v>44819</v>
+      </c>
+      <c r="B179" t="n">
+        <v>1</v>
+      </c>
+      <c r="C179" t="n">
+        <v>1</v>
+      </c>
+      <c r="D179" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="n">
+        <v>44820</v>
+      </c>
+      <c r="B180" t="n">
+        <v>1</v>
+      </c>
+      <c r="C180" t="n">
+        <v>1</v>
+      </c>
+      <c r="D180" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="n">
+        <v>44823</v>
+      </c>
+      <c r="B181" t="n">
+        <v>1</v>
+      </c>
+      <c r="C181" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="n">
+        <v>44824</v>
+      </c>
+      <c r="B182" t="n">
+        <v>1</v>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="n">
+        <v>44825</v>
+      </c>
+      <c r="B183" t="n">
+        <v>1</v>
+      </c>
+      <c r="C183" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="n">
+        <v>44826</v>
+      </c>
+      <c r="B184" t="n">
+        <v>1</v>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="n">
+        <v>44827</v>
+      </c>
+      <c r="B185" t="n">
+        <v>1</v>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n">
+        <v>44830</v>
+      </c>
+      <c r="B186" t="n">
+        <v>1</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="n">
+        <v>44831</v>
+      </c>
+      <c r="B187" t="n">
+        <v>1</v>
+      </c>
+      <c r="C187" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="n">
+        <v>44832</v>
+      </c>
+      <c r="B188" t="n">
+        <v>1</v>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="n">
+        <v>44833</v>
+      </c>
+      <c r="B189" t="n">
+        <v>1</v>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="n">
+        <v>44834</v>
+      </c>
+      <c r="B190" t="n">
+        <v>1</v>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="n">
+        <v>44837</v>
+      </c>
+      <c r="B191" t="n">
+        <v>1</v>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="n">
+        <v>44838</v>
+      </c>
+      <c r="B192" t="n">
+        <v>1</v>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="n">
+        <v>44839</v>
+      </c>
+      <c r="B193" t="n">
+        <v>1</v>
+      </c>
+      <c r="C193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="n">
+        <v>44840</v>
+      </c>
+      <c r="B194" t="n">
+        <v>1</v>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="n">
+        <v>44841</v>
+      </c>
+      <c r="B195" t="n">
+        <v>1</v>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="n">
+        <v>44844</v>
+      </c>
+      <c r="B196" t="n">
+        <v>1</v>
+      </c>
+      <c r="C196" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="n">
+        <v>44845</v>
+      </c>
+      <c r="B197" t="n">
+        <v>1</v>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="n">
+        <v>44847</v>
+      </c>
+      <c r="B198" t="n">
+        <v>1</v>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="n">
+        <v>44848</v>
+      </c>
+      <c r="B199" t="n">
+        <v>1</v>
+      </c>
+      <c r="C199" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="n">
+        <v>44851</v>
+      </c>
+      <c r="B200" t="n">
+        <v>1</v>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="n">
+        <v>44852</v>
+      </c>
+      <c r="B201" t="n">
+        <v>1</v>
+      </c>
+      <c r="C201" t="n">
+        <v>1</v>
+      </c>
+      <c r="D201" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="n">
+        <v>44853</v>
+      </c>
+      <c r="B202" t="n">
+        <v>1</v>
+      </c>
+      <c r="C202" t="n">
+        <v>1</v>
+      </c>
+      <c r="D202" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="n">
+        <v>44854</v>
+      </c>
+      <c r="B203" t="n">
+        <v>1</v>
+      </c>
+      <c r="C203" t="n">
+        <v>1</v>
+      </c>
+      <c r="D203" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="n">
+        <v>44855</v>
+      </c>
+      <c r="B204" t="n">
+        <v>1</v>
+      </c>
+      <c r="C204" t="n">
+        <v>1</v>
+      </c>
+      <c r="D204" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="n">
+        <v>44858</v>
+      </c>
+      <c r="B205" t="n">
+        <v>1</v>
+      </c>
+      <c r="C205" t="n">
+        <v>1</v>
+      </c>
+      <c r="D205" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="n">
+        <v>44859</v>
+      </c>
+      <c r="B206" t="n">
+        <v>1</v>
+      </c>
+      <c r="C206" t="n">
+        <v>1</v>
+      </c>
+      <c r="D206" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="n">
+        <v>44860</v>
+      </c>
+      <c r="B207" t="n">
+        <v>1</v>
+      </c>
+      <c r="C207" t="n">
+        <v>1</v>
+      </c>
+      <c r="D207" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="n">
+        <v>44861</v>
+      </c>
+      <c r="B208" t="n">
+        <v>1</v>
+      </c>
+      <c r="C208" t="n">
+        <v>1</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="n">
+        <v>44862</v>
+      </c>
+      <c r="B209" t="n">
+        <v>1</v>
+      </c>
+      <c r="C209" t="n">
+        <v>1</v>
+      </c>
+      <c r="D209" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="n">
+        <v>44865</v>
+      </c>
+      <c r="B210" t="n">
+        <v>1</v>
+      </c>
+      <c r="C210" t="n">
+        <v>1</v>
+      </c>
+      <c r="D210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="n">
+        <v>44866</v>
+      </c>
+      <c r="B211" t="n">
+        <v>1</v>
+      </c>
+      <c r="C211" t="n">
+        <v>1</v>
+      </c>
+      <c r="D211" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="n">
+        <v>44868</v>
+      </c>
+      <c r="B212" t="n">
+        <v>1</v>
+      </c>
+      <c r="C212" t="n">
+        <v>1</v>
+      </c>
+      <c r="D212" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="n">
+        <v>44869</v>
+      </c>
+      <c r="B213" t="n">
+        <v>1</v>
+      </c>
+      <c r="C213" t="n">
+        <v>1</v>
+      </c>
+      <c r="D213" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="n">
+        <v>44872</v>
+      </c>
+      <c r="B214" t="n">
+        <v>1</v>
+      </c>
+      <c r="C214" t="n">
+        <v>1</v>
+      </c>
+      <c r="D214" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="n">
+        <v>44873</v>
+      </c>
+      <c r="B215" t="n">
+        <v>1</v>
+      </c>
+      <c r="C215" t="n">
+        <v>1</v>
+      </c>
+      <c r="D215" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="n">
+        <v>44874</v>
+      </c>
+      <c r="B216" t="n">
+        <v>1</v>
+      </c>
+      <c r="C216" t="n">
+        <v>1</v>
+      </c>
+      <c r="D216" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="n">
+        <v>44875</v>
+      </c>
+      <c r="B217" t="n">
+        <v>1</v>
+      </c>
+      <c r="C217" t="n">
+        <v>1</v>
+      </c>
+      <c r="D217" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="n">
+        <v>44876</v>
+      </c>
+      <c r="B218" t="n">
+        <v>1</v>
+      </c>
+      <c r="C218" t="n">
+        <v>1</v>
+      </c>
+      <c r="D218" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="n">
+        <v>44879</v>
+      </c>
+      <c r="B219" t="n">
+        <v>1</v>
+      </c>
+      <c r="C219" t="n">
+        <v>1</v>
+      </c>
+      <c r="D219" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="n">
+        <v>44881</v>
+      </c>
+      <c r="B220" t="n">
+        <v>1</v>
+      </c>
+      <c r="C220" t="n">
+        <v>1</v>
+      </c>
+      <c r="D220" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="n">
+        <v>44882</v>
+      </c>
+      <c r="B221" t="n">
+        <v>1</v>
+      </c>
+      <c r="C221" t="n">
+        <v>1</v>
+      </c>
+      <c r="D221" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n">
+        <v>44883</v>
+      </c>
+      <c r="B222" t="n">
+        <v>1</v>
+      </c>
+      <c r="C222" t="n">
+        <v>1</v>
+      </c>
+      <c r="D222" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n">
+        <v>44886</v>
+      </c>
+      <c r="B223" t="n">
+        <v>1</v>
+      </c>
+      <c r="C223" t="n">
+        <v>1</v>
+      </c>
+      <c r="D223" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n">
+        <v>44887</v>
+      </c>
+      <c r="B224" t="n">
+        <v>1</v>
+      </c>
+      <c r="C224" t="n">
+        <v>1</v>
+      </c>
+      <c r="D224" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n">
+        <v>44888</v>
+      </c>
+      <c r="B225" t="n">
+        <v>1</v>
+      </c>
+      <c r="C225" t="n">
+        <v>1</v>
+      </c>
+      <c r="D225" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n">
+        <v>44889</v>
+      </c>
+      <c r="B226" t="n">
+        <v>1</v>
+      </c>
+      <c r="C226" t="n">
+        <v>1</v>
+      </c>
+      <c r="D226" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n">
+        <v>44890</v>
+      </c>
+      <c r="B227" t="n">
+        <v>1</v>
+      </c>
+      <c r="C227" t="n">
+        <v>1</v>
+      </c>
+      <c r="D227" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n">
+        <v>44893</v>
+      </c>
+      <c r="B228" t="n">
+        <v>1</v>
+      </c>
+      <c r="C228" t="n">
+        <v>1</v>
+      </c>
+      <c r="D228" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n">
+        <v>44894</v>
+      </c>
+      <c r="B229" t="n">
+        <v>1</v>
+      </c>
+      <c r="C229" t="n">
+        <v>1</v>
+      </c>
+      <c r="D229" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n">
+        <v>44895</v>
+      </c>
+      <c r="B230" t="n">
+        <v>1</v>
+      </c>
+      <c r="C230" t="n">
+        <v>1</v>
+      </c>
+      <c r="D230" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n">
+        <v>44896</v>
+      </c>
+      <c r="B231" t="n">
+        <v>1</v>
+      </c>
+      <c r="C231" t="n">
+        <v>1</v>
+      </c>
+      <c r="D231" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n">
+        <v>44897</v>
+      </c>
+      <c r="B232" t="n">
+        <v>1</v>
+      </c>
+      <c r="C232" t="n">
+        <v>1</v>
+      </c>
+      <c r="D232" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n">
+        <v>44900</v>
+      </c>
+      <c r="B233" t="n">
+        <v>1</v>
+      </c>
+      <c r="C233" t="n">
+        <v>1</v>
+      </c>
+      <c r="D233" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n">
+        <v>44901</v>
+      </c>
+      <c r="B234" t="n">
+        <v>1</v>
+      </c>
+      <c r="C234" t="n">
+        <v>1</v>
+      </c>
+      <c r="D234" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n">
+        <v>44902</v>
+      </c>
+      <c r="B235" t="n">
+        <v>1</v>
+      </c>
+      <c r="C235" t="n">
+        <v>1</v>
+      </c>
+      <c r="D235" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n">
+        <v>44903</v>
+      </c>
+      <c r="B236" t="n">
+        <v>1</v>
+      </c>
+      <c r="C236" t="n">
+        <v>1</v>
+      </c>
+      <c r="D236" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n">
+        <v>44904</v>
+      </c>
+      <c r="B237" t="n">
+        <v>1</v>
+      </c>
+      <c r="C237" t="n">
+        <v>1</v>
+      </c>
+      <c r="D237" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n">
+        <v>44907</v>
+      </c>
+      <c r="B238" t="n">
+        <v>1</v>
+      </c>
+      <c r="C238" t="n">
+        <v>1</v>
+      </c>
+      <c r="D238" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n">
+        <v>44908</v>
+      </c>
+      <c r="B239" t="n">
+        <v>1</v>
+      </c>
+      <c r="C239" t="n">
+        <v>1</v>
+      </c>
+      <c r="D239" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n">
+        <v>44909</v>
+      </c>
+      <c r="B240" t="n">
+        <v>1</v>
+      </c>
+      <c r="C240" t="n">
+        <v>1</v>
+      </c>
+      <c r="D240" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n">
+        <v>44910</v>
+      </c>
+      <c r="B241" t="n">
+        <v>1</v>
+      </c>
+      <c r="C241" t="n">
+        <v>1</v>
+      </c>
+      <c r="D241" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n">
+        <v>44911</v>
+      </c>
+      <c r="B242" t="n">
+        <v>1</v>
+      </c>
+      <c r="C242" t="n">
+        <v>1</v>
+      </c>
+      <c r="D242" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n">
+        <v>44914</v>
+      </c>
+      <c r="B243" t="n">
+        <v>1</v>
+      </c>
+      <c r="C243" t="n">
+        <v>1</v>
+      </c>
+      <c r="D243" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n">
+        <v>44915</v>
+      </c>
+      <c r="B244" t="n">
+        <v>1</v>
+      </c>
+      <c r="C244" t="n">
+        <v>1</v>
+      </c>
+      <c r="D244" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n">
+        <v>44916</v>
+      </c>
+      <c r="B245" t="n">
+        <v>1</v>
+      </c>
+      <c r="C245" t="n">
+        <v>1</v>
+      </c>
+      <c r="D245" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n">
+        <v>44917</v>
+      </c>
+      <c r="B246" t="n">
+        <v>1</v>
+      </c>
+      <c r="C246" t="n">
+        <v>1</v>
+      </c>
+      <c r="D246" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n">
+        <v>44918</v>
+      </c>
+      <c r="B247" t="n">
+        <v>1</v>
+      </c>
+      <c r="C247" t="n">
+        <v>1</v>
+      </c>
+      <c r="D247" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n">
+        <v>44921</v>
+      </c>
+      <c r="B248" t="n">
+        <v>1</v>
+      </c>
+      <c r="C248" t="n">
+        <v>1</v>
+      </c>
+      <c r="D248" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n">
+        <v>44922</v>
+      </c>
+      <c r="B249" t="n">
+        <v>1</v>
+      </c>
+      <c r="C249" t="n">
+        <v>1</v>
+      </c>
+      <c r="D249" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n">
+        <v>44923</v>
+      </c>
+      <c r="B250" t="n">
+        <v>1</v>
+      </c>
+      <c r="C250" t="n">
+        <v>1</v>
+      </c>
+      <c r="D250" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n">
+        <v>44924</v>
+      </c>
+      <c r="B251" t="n">
+        <v>1</v>
+      </c>
+      <c r="C251" t="n">
+        <v>1</v>
+      </c>
+      <c r="D251" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>